<commit_message>
feat: repo + tooling (Day 2)
Scaffold Next.js 16 (Turbopack) + TypeScript + ESLint (App Router,
src dir, @/* alias). Add Prettier (with eslint-config-prettier),
Husky pre-commit running lint-staged, .env.example for DATABASE_URL,
and a README documenting scripts and git workflow. Verified: fresh
install, lint, and build all pass locally.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -590,10 +590,14 @@
       </c>
       <c r="I3" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J3" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J3" s="11" t="inlineStr">
+        <is>
+          <t>Next.js 16 (Turbopack) + TS + ESLint scaffolded, plus Prettier, Husky pre-commit (lint-staged), .env.example, README with git-workflow notes. lint/build verified locally.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="9">
       <c r="A4" s="11" t="n">
@@ -7957,10 +7961,12 @@
       <c r="C3" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="11" t="n"/>
+      <c r="D3" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E3" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F3" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: database - PostgreSQL + Prisma (Day 4)
Wire up Prisma 7 against PostgreSQL via the pg driver adapter
(@prisma/adapter-pg) - Prisma 7 no longer takes a datasource url in
schema.prisma, so the connection lives in prisma7.config.ts (for
Migrate) and the adapter (for the client), per src/modules/kernel/db.ts.

Local dev DB is `npx prisma dev` (an embedded PGlite Postgres) since
Docker Desktop wouldn't come up in this sandbox. Note for later:
PGlite doesn't support native Postgres extensions - a pgcrypto
migration failed - so ID generation should stay on Prisma's own
uuid()/cuid() defaults rather than DB extensions, for portability
between PGlite and real Postgres.

Verified with a real automated test (src/modules/kernel/db.test.ts)
that runs a live query against the dev database, plus lint/build.
No domain models yet - Core schema is Day 5.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -686,10 +686,14 @@
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Prisma 7 + PostgreSQL wired up via the pg driver adapter (schema.prisma has no url field in Prisma 7 - connection lives in prisma7.config.ts + the adapter). Local dev DB is npx prisma dev (embedded PGlite Postgres, no Docker needed - Docker Desktop would not start in this sandbox). Note: PGlite does not support native extensions (pgcrypto attempt failed) - stick to Prisma-side ID generation (uuid()/cuid()), not DB extensions, for portability. Kernel db client (src/modules/kernel/db.ts) added with a passing automated test that runs a real query against the live dev DB. No domain models yet - that is Day 5.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="55.2" customHeight="1" s="9">
       <c r="A6" s="11" t="n">
@@ -8013,10 +8017,12 @@
       <c r="C5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="11" t="n"/>
+      <c r="D5" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F5" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: core schema - Organisation, Department, Role, User (Day 5)
Add the four base Identity models per docs/ARCHITECTURE.md, designed
multi-tenant-ready from day one: Organisation is the tenant root,
and Department/Role/User all carry organisationId with cascade
delete and a per-organisation uniqueness constraint on name/email.
IDs use Prisma's uuid() default rather than a Postgres extension
(see Day 4's PGlite note).

5 automated tests (src/modules/identity/schema.test.ts) cover
create/read across the model graph, relation loading, duplicate-name
rejection, and cascade delete on the organisation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -734,10 +734,14 @@
       </c>
       <c r="I6" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>Organisation, Department, Role, User models in prisma/schema.prisma (migration 20260918094921_core_schema). Organisation is the tenant root (no org_id on itself); Department/Role/User all carry organisationId with cascade delete, plus a unique(organisationId, name/email) constraint. IDs are Prisma-generated UUIDs (not a DB extension - see Day 4 note). department/roleId on User are nullable at the DB level; Day 20 (Create employee) will decide whether to require them at the validation layer. 5 automated tests in src/modules/identity/schema.test.ts cover create/read, relations, duplicate-name rejection, and cascade delete.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="9">
       <c r="A7" s="11" t="n">
@@ -8041,10 +8045,12 @@
       <c r="C6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="11" t="n"/>
+      <c r="D6" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F6" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: validation + error conventions (Day 6)
Add the shared API error convention: ApiError + toApiErrorResponse()
(src/modules/kernel/errors.ts) map an ApiError, a zod ValidationError,
or anything unexpected to one predictable JSON shape
({ error: { code, message, details? } }) with the right status code,
and never leak internal error messages for unexpected failures.

zod is the shared validation library. POST /api/health/echo is the
reference implementation of the validate-then-respond pattern every
future route handler should follow. 6 automated tests cover a valid
payload, a validation failure, and malformed JSON.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -782,10 +782,14 @@
       </c>
       <c r="I7" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Shared ApiError class + toApiErrorResponse() (src/modules/kernel/errors.ts) map ApiError/ZodError/unknown errors to one predictable {error:{code,message,details?}} JSON shape. zod is the standard validation library. Reference implementation wired into a new POST /api/health/echo route (validate-then-respond pattern every future route copies). 6 automated tests cover valid payload, validation failure, and malformed JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="9">
       <c r="A8" s="11" t="n">
@@ -8069,10 +8073,12 @@
       <c r="C7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="11" t="n"/>
+      <c r="D7" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F7" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: UI shell (Day 7)
Add AppShell (src/components/AppShell.tsx): a sticky header and an
off-canvas sidebar nav that's always visible at >=768px and toggled
by a menu button below that, per CLAUDE.md's mobile-friendly
principle. Wired into the root layout; replaced the default
create-next-app starter homepage with a placeholder dashboard.
Playwright covers both a desktop and a mobile viewport
(e2e/app-shell.spec.ts).

Also fixes a real flakiness bug surfaced while testing this: Vitest
running test files in parallel was destabilizing connections to the
PGlite dev database ("Connection terminated unexpectedly",
intermittent). Fixed with fileParallelism: false, a pool size cap,
and explicit $disconnect() in afterAll for tests that touch the db.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -830,10 +830,14 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>AppShell component (src/components/AppShell.tsx): sticky header + off-canvas sidebar nav, CSS-media-query responsive (sidebar always visible &gt;=768px, toggled via a menu button below that). Replaced the default create-next-app starter homepage. Also fixed a real flakiness bug found while testing this: Vitest running test files in parallel was destabilizing the PGlite dev DB connection (fileParallelism disabled + pool max + explicit  in db-touching tests - see dev_environment memory). Playwright desktop+mobile viewport smoke test in e2e/app-shell.spec.ts, both passing.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="9">
       <c r="A9" s="11" t="n">
@@ -8097,10 +8101,12 @@
       <c r="C8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="11" t="n"/>
+      <c r="D8" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: observability - structured logging (Day 8)
Add structured JSON logging via pino (src/modules/kernel/logging.ts,
pretty-printed in dev only). Wire it into the shared error handler
from Day 6: unexpected errors log at error level with the full
error, handled ApiErrors log at warn level (code + status only).
Every route already following the Day 6 convention gets this for
free - no per-route logging code needed.

2 automated tests: pino emits a structured JSON line with the
expected fields, and the error handler actually invokes the logger
when it handles an unexpected error.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -878,10 +878,14 @@
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>Structured JSON logging via pino (src/modules/kernel/logging.ts, pino-pretty in dev only). Wired into the shared error handler from Day 6: toApiErrorResponse() logs unexpected errors at error level (with the full error object) and handled ApiErrors at warn level (code + status, no stack noise) - so every route that already follows the Day 6 convention gets logging for free with no extra code. 2 automated tests: one verifies pino emits a structured JSON line with level/time/msg/fields, one verifies the error handler actually calls the logger on an unexpected error.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="9">
       <c r="A10" s="11" t="n">
@@ -8125,10 +8129,12 @@
       <c r="C9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="11" t="n"/>
+      <c r="D9" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F9" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: seed data (Day 9)
Add an idempotent dev seed (prisma/seed-data.ts: seedDatabase(),
all upserts) - one organisation, 3 departments, 3 roles, 1 owner
user. Wired via prisma7.config.ts's migrations.seed using tsx
(plain `node --experimental-strip-types` can't resolve the @/*
tsconfig path alias used everywhere else). `npm run db:seed` runs
it. Verified idempotent locally (ran twice, no errors/duplicates).

2 automated tests (prisma/seed-data.test.ts) cover the happy path
and re-running without duplication.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -926,10 +926,14 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>Idempotent seed (prisma/seed-data.ts: seedDatabase(), all upserts) seeding one organisation, 3 departments, 3 roles, 1 owner user. Wired via prisma7.config.ts migrations.seed using tsx (plain node --experimental-strip-types could not resolve the @/* tsconfig path alias). npm run db:seed -&gt; prisma db seed. Verified idempotent by running twice locally with no errors/duplicates. 2 automated tests (prisma/seed-data.test.ts) cover the happy path and re-running without duplication.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="28.35" customHeight="1" s="9">
       <c r="A11" s="11" t="n">
@@ -8153,10 +8157,12 @@
       <c r="C10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="11" t="n"/>
+      <c r="D10" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F10" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: CI pipeline (Day 10)
Add .github/workflows/ci.yml: on every push/PR (any branch), spin
up a Postgres 16 service container, npm ci, apply migrations, then
lint, typecheck, format:check, vitest, build, and Playwright e2e
(ubuntu-latest ships Chrome, matching the channel: "chrome" config
from Day 3's Playwright setup).

This closes out the Foundation phase (Days 1-10): architecture,
repo/tooling, test harness, database, core schema, validation/error
conventions, UI shell, observability, seed data, and now CI.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -974,10 +974,14 @@
       </c>
       <c r="I11" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="n"/>
+          <t>Done (pending first push to verify green)</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>.github/workflows/ci.yml: on push/PR to any branch, a Postgres 16 service container, npm ci, prisma migrate deploy, lint, typecheck, format:check, vitest, build, then Playwright e2e (ubuntu-latest ships Chrome, matching the channel:"chrome" config from Day 3). YAML validated locally. The literal acceptance check (a deliberately-broken test fails the pipeline, a passing one goes green) needs an actual push to github.com/SakshiK2503/ai-firm-management to observe - the repo has a configured origin remote but nothing has been pushed yet this session; flagged to the founder rather than pushed without asking.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="9">
       <c r="A12" s="11" t="n">
@@ -8181,10 +8185,12 @@
       <c r="C11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="11" t="n"/>
+      <c r="D11" s="11" t="n">
+        <v>1</v>
+      </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done (pending push)</t>
         </is>
       </c>
       <c r="F11" s="11" t="n"/>

</xml_diff>

<commit_message>
feat: manager/reporting hierarchy (Day 24)
Self-referential managerId on User, with service-layer cycle prevention
(direct self-management and any longer reporting chain). Surfaced on the
employee create/edit forms and detail page, replacing the Day 22 "not
tracked yet" placeholder.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -439,7 +439,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:J168"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="8" min="1" max="2"/>
     <col width="28" customWidth="1" style="8" min="3" max="4"/>
@@ -1646,10 +1646,14 @@
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J25" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
+        <is>
+          <t>Migration adds self-referential managerId/manager/directReports on User (nullable - not every employee has a manager). employee.service.ts: assertManagerAssignable() rejects an unknown/cross-org manager, direct self-management (managerId === own id), and any longer cycle (walks up the proposed manager's own chain looking for the employee being updated). Wired into both createEmployee (optional managerId) and updateEmployee (managerId?: string | null - null clears it, omitted leaves it untouched). Employee detail page now shows the real manager (replacing Day 22's "Not tracked yet" placeholder) with a link to their profile, plus a manager select on both the create and edit forms. 6 new unit/service tests (assign, clear, unknown manager, self-management, 2-node cycle, 3-node cycle) + 3 new API route tests + 1 new Playwright E2E test (assign a manager, then verify a cycle attempt is rejected with the correct message).</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="9">
       <c r="A26" s="11" t="n">
@@ -7965,7 +7969,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:F103"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="8" min="1" max="1"/>
     <col width="34" customWidth="1" style="8" min="2" max="2"/>
@@ -8453,13 +8457,19 @@
       <c r="C20" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D20" s="11" t="n"/>
+      <c r="D20" s="11" t="n">
+        <v>24</v>
+      </c>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F20" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Self-referential manager relationship with cycle prevention (see Daily Plan Day 24).</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="9">
       <c r="A21" s="11" t="inlineStr">
@@ -10302,7 +10312,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:G35"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="8" min="1" max="1"/>
     <col width="12" customWidth="1" style="8" min="2" max="2"/>
@@ -11384,7 +11394,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="8" min="1" max="1"/>
     <col width="15" customWidth="1" style="8" min="2" max="2"/>
@@ -11590,7 +11600,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="8" min="1" max="1"/>
     <col width="110" customWidth="1" style="8" min="2" max="2"/>
@@ -11714,7 +11724,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="28" customWidth="1" style="8" min="1" max="1"/>
     <col width="20" customWidth="1" style="8" min="2" max="2"/>
@@ -11801,7 +11811,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D39"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="48" customWidth="1" style="8" min="1" max="2"/>
     <col width="14" customWidth="1" style="8" min="3" max="3"/>
@@ -12681,7 +12691,7 @@
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
   <dimension ref="A1:D14"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="8" min="1" max="1"/>
     <col width="58" customWidth="1" style="8" min="2" max="2"/>

</xml_diff>

<commit_message>
feat: service master - hierarchy, lifecycle, checklist (Days 37-41)
Adds the Service catalogue: org-scoped services with a self-referential
parent/child hierarchy (cycle-safe, mirrors the Day 24 manager pattern),
department + expected-skill-level requirements, edit/disable lifecycle
(assertServiceAssignable blocks new assignment of a disabled service,
ready for Day 35's Engagement work), and a reusable checklist template
per service. Unblocks Day 35 (Engagements), previously marked Blocked
since its own acceptance check depends on Service existing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J200"/>
+  <dimension ref="A1:J168"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="8" min="1" max="2"/>
@@ -2174,12 +2174,12 @@
       </c>
       <c r="I36" s="11" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="J36" s="11" t="inlineStr">
         <is>
-          <t>BLOCKED: this row's own acceptance check is 'Service linked to entity/client', but Service doesn't exist yet - Service Master is Days 37-41, later in the same Daily Plan. An Engagement literally cannot be built to spec without something to link to. Per CLAUDE.md: 'don't silently carry it forward or weaken the test to make it pass' - flagging this rather than either skipping silently or building a fake/placeholder service link. Plan: build Service Master (Days 37-41) next, then come straight back to complete this row against the real Service model.</t>
+          <t>Unblocked: Service Master (Days 37-41) is now built. Ready to build the Engagement model linking a ClientEntity to a Service, per this row's acceptance check.</t>
         </is>
       </c>
     </row>
@@ -2270,10 +2270,14 @@
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J38" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J38" s="11" t="inlineStr">
+        <is>
+          <t>Service model created (name, org-scoped), createService with required-metadata validation and duplicate-name-per-parent rejection. API: POST/GET /api/services. Unit/API tests cover happy path, validation error, permission (403 Preparer), and auth (401 logged out).</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="9">
       <c r="A39" s="11" t="n">
@@ -2314,10 +2318,14 @@
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J39" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J39" s="11" t="inlineStr">
+        <is>
+          <t>Self-referential Service.parentId with cycle prevention (assertParentValid walks up from proposed parent) mirroring the Day 24 manager-hierarchy pattern. listServiceTree returns a nested children[] tree; UI renders it indented and recursively. Tests cover nesting, self-parent rejection, and circular-parent rejection.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="9">
       <c r="A40" s="11" t="n">
@@ -2358,10 +2366,14 @@
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J40" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J40" s="11" t="inlineStr">
+        <is>
+          <t>updateService supports isActive toggle (Disable/Enable in UI); assertServiceAssignable throws SERVICE_DISABLED for a disabled service, ready for Engagement (Day 35) to consume. Tests cover disable, the assignability check failing while disabled, and re-enabling.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="9">
       <c r="A41" s="11" t="n">
@@ -2402,10 +2414,14 @@
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J41" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>Service.departmentId (FK to Department, validated) and Service.expectedSkillLevel (SkillLevel enum) stored and returned via getService/listServiceTree/updateService; set and edited from the Service create form and detail-page edit form. Covered by the Day 37 create test (department + skill level asserted on the created record) and the Day 39 update tests.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="9">
       <c r="A42" s="11" t="n">
@@ -2446,10 +2462,14 @@
       </c>
       <c r="I42" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J42" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr">
+        <is>
+          <t>ChecklistTemplate (1:1 with Service, @@unique serviceId) + ChecklistItem models; checklist.service.ts creates a template with its starting items in one call, and supports add/remove items. API: GET/POST /api/services/[id]/checklist, POST items, DELETE items/[itemId]. UI: ServiceChecklist.tsx on the service detail page. Tests cover empty state, template creation, rejecting a second template (409), rejecting an empty item list, adding/removing items, and a 404 when adding an item before any template exists.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="9">
       <c r="A43" s="11" t="n">
@@ -7988,38 +8008,6 @@
         </is>
       </c>
     </row>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
   </sheetData>
   <autoFilter ref="A1:J161"/>
   <conditionalFormatting sqref="I2:I161">
@@ -8048,7 +8036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="8" min="1" max="1"/>
@@ -8708,12 +8696,12 @@
       <c r="D26" s="11" t="n"/>
       <c r="E26" s="11" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Not Started</t>
         </is>
       </c>
       <c r="F26" s="11" t="inlineStr">
         <is>
-          <t>Needs Service Master (Days 37-41) to exist first - see Daily Plan Day 35.</t>
+          <t>Unblocked now that Service Master exists (Daily Plan Days 37-41) - ready to build against the real Service model (see Daily Plan Day 35).</t>
         </is>
       </c>
     </row>
@@ -8759,13 +8747,19 @@
       <c r="C28" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D28" s="11" t="n"/>
+      <c r="D28" s="11" t="n">
+        <v>39</v>
+      </c>
       <c r="E28" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F28" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Service model with required metadata, parent-child hierarchy (cycle-safe), and edit/disable lifecycle (see Daily Plan Days 37-39).</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="9">
       <c r="A29" s="11" t="inlineStr">
@@ -8781,13 +8775,19 @@
       <c r="C29" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="D29" s="11" t="n"/>
+      <c r="D29" s="11" t="n">
+        <v>41</v>
+      </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F29" s="11" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Department + expected skill level requirements, and a reusable checklist template attached per service, are done (Daily Plan Days 40-41). TAT/effort/reviewer defaults (Day 42) not yet built.</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="9">
       <c r="A30" s="11" t="inlineStr">
@@ -10411,103 +10411,6 @@
         </is>
       </c>
     </row>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
-    <row r="108"/>
-    <row r="109"/>
-    <row r="110"/>
-    <row r="111"/>
-    <row r="112"/>
-    <row r="113"/>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
-    <row r="131"/>
-    <row r="132"/>
-    <row r="133"/>
-    <row r="134"/>
-    <row r="135"/>
-    <row r="136"/>
-    <row r="137"/>
-    <row r="138"/>
-    <row r="139"/>
-    <row r="140"/>
-    <row r="141"/>
-    <row r="142"/>
-    <row r="143"/>
-    <row r="144"/>
-    <row r="145"/>
-    <row r="146"/>
-    <row r="147"/>
-    <row r="148"/>
-    <row r="149"/>
-    <row r="150"/>
-    <row r="151"/>
-    <row r="152"/>
-    <row r="153"/>
-    <row r="154"/>
-    <row r="155"/>
-    <row r="156"/>
-    <row r="157"/>
-    <row r="158"/>
-    <row r="159"/>
-    <row r="160"/>
-    <row r="161"/>
-    <row r="162"/>
-    <row r="163"/>
-    <row r="164"/>
-    <row r="165"/>
-    <row r="166"/>
-    <row r="167"/>
-    <row r="168"/>
-    <row r="169"/>
-    <row r="170"/>
-    <row r="171"/>
-    <row r="172"/>
-    <row r="173"/>
-    <row r="174"/>
-    <row r="175"/>
-    <row r="176"/>
-    <row r="177"/>
-    <row r="178"/>
-    <row r="179"/>
-    <row r="180"/>
-    <row r="181"/>
-    <row r="182"/>
-    <row r="183"/>
-    <row r="184"/>
-    <row r="185"/>
-    <row r="186"/>
-    <row r="187"/>
-    <row r="188"/>
-    <row r="189"/>
-    <row r="190"/>
-    <row r="191"/>
-    <row r="192"/>
-    <row r="193"/>
-    <row r="194"/>
-    <row r="195"/>
-    <row r="196"/>
-    <row r="197"/>
-    <row r="198"/>
-    <row r="199"/>
-    <row r="200"/>
   </sheetData>
   <autoFilter ref="A1:F100"/>
   <dataValidations count="1">

</xml_diff>

<commit_message>
feat: service defaults and recurring configuration (Days 42-43)
Day 42 - TAT/effort/reviewer defaults were already stored on Service
(Days 37-41), but the create/edit UI never exposed the effort range or
standard documents fields (API-only). Closes that gap, plus a new
cross-field rule: estimated effort max must be >= min, checked on both
create and partial update.

Day 43 - RecurringConfig (frequency + day/month, PRD S32), one per
recurring Service. computeNextOccurrence is a pure, unit-tested
function - "generate a test recurring instance" is literally calling
it, since generating an actual Task from it is Task Engine's job
(Day 44+), same pattern as Day 41's checklist template being just the
template. UI lets a Partner configure the calendar and preview the
next occurrence, shown only when a service is marked recurring.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -2510,10 +2510,14 @@
       </c>
       <c r="I43" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J43" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J43" s="11" t="inlineStr">
+        <is>
+          <t>TAT/effort/reviewer defaults (turnaroundDays, estimatedEffortMinHours/MaxHours, reviewRequired) were already stored via the Day 37-41 Service model, but the create/edit UI forms did not expose the effort range or standardDocuments fields (API-only). Closed that gap: both fields now on ServicesAdmin.tsx (create) and ServiceDetail.tsx (edit), plus a new cross-field rule (estimatedEffortMaxHours must be &gt;= estimatedEffortMinHours, checked on both create and partial update) since an inverted range is invalid data, not a valid one. Unit/API + E2E tests cover the full round trip and the rejection.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="9">
       <c r="A44" s="11" t="n">
@@ -2554,10 +2558,14 @@
       </c>
       <c r="I44" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J44" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J44" s="11" t="inlineStr">
+        <is>
+          <t>New RecurringConfig model (1:1 with a recurring Service): frequency (Monthly/Quarterly/Annually, PRD S32) + dayOfMonth (capped 1-28) + monthOfYear (Annually only). computeNextOccurrence is a pure, unit-tested function - "generate a test recurring instance" is literally calling it, since actually generating a Task from it is Task Engine's job (Day 44+), same pattern as Day 41's checklist template being just the template. API + UI (service detail page, shown only when isRecurring) let a Partner set the calendar and preview the next occurrence. Gated on service:manage to configure, service:view to see it.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="9">
       <c r="A45" s="11" t="n">
@@ -8778,16 +8786,16 @@
         <v>3</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E29" s="11" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="11" t="inlineStr">
         <is>
-          <t>Department + expected skill level requirements, and a reusable checklist template attached per service, are done (Daily Plan Days 40-41). TAT/effort/reviewer defaults (Day 42) not yet built.</t>
+          <t>Department + skill requirements, standard checklist, and TAT/effort/reviewer defaults - all on the Service model (see Daily Plan Days 40-42).</t>
         </is>
       </c>
     </row>
@@ -8805,13 +8813,19 @@
       <c r="C30" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D30" s="11" t="n"/>
+      <c r="D30" s="11" t="n">
+        <v>43</v>
+      </c>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F30" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Recurrence calendar (frequency + day/month) per recurring service, with a next-occurrence computation baseline for Task Engine to consume later (see Daily Plan Day 43).</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="9">
       <c r="A31" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat: task list filters - status, client, priority (Day 46)
Adds status/client/priority filters (query params, validated) to
GET /api/tasks and a filter bar on the Tasks page, with a "Clear
filters" reset.

PARTIALLY DONE by design: this row's own acceptance check also lists
an assignee filter and a date filter, but neither has a backing field
yet - assignedToId is Assignment's day (49), dueDate is Dates' day
(51). Both will extend this same route/filter bar once those land,
not guessed at now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -2702,10 +2702,14 @@
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J47" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J47" s="11" t="inlineStr">
+        <is>
+          <t>Filters implemented for status, client, and priority (query params, validated). PARTIALLY DONE by design: this row also lists an assignee filter and a date filter, but neither has a backing field yet (assignedToId is Assignment/Day 49, dueDate is Dates/Day 51) - both will be added to this same GET /api/tasks route + filter bar once those days land, not guessed at now. Same task:viewAll/assigned scoping as task list itself (empty for a Preparer today, same known gap as Client). Unit/API + E2E tests cover each filter and an invalid filter value.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="9">
       <c r="A48" s="11" t="n">
@@ -8877,13 +8881,19 @@
       <c r="C32" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D32" s="11" t="n"/>
+      <c r="D32" s="11" t="n">
+        <v>46</v>
+      </c>
       <c r="E32" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F32" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Task queue with status/client/priority filters; assignee/date filters follow once Assignment (Day 49) and Dates (Day 51) add their fields (see Daily Plan Day 46).</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="9">
       <c r="A33" s="11" t="inlineStr">

</xml_diff>

<commit_message>
feat: task detail workspace (Day 47)
Adds /tasks/[id] and GET /api/tasks/[id] (same route pattern as
Client/Entity/Service). Shows Core task fields plus related data that
already exists: the Engagement for this task's entity/service pairing
(billing structure, start date, active/terminated), fetched
separately to demonstrate real related-data loading rather than just
the task row's own denormalized fields.

PRD S18 describes a much larger detail screen (Client Instruction, AI
Interpretation, Checklist, Attachments, Working Papers, Time,
Comments, Client Communication, Review, Activity Timeline) - almost
none of which exists yet, since those are separate later days/phases
(AI intake, attachments, time tracking, comments, review, activity
log). This page grows one section at a time as each of those days
lands, rather than stubbing placeholders now.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap.xlsx
+++ b/docs/roadmap.xlsx
@@ -2750,10 +2750,14 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="J48" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J48" s="11" t="inlineStr">
+        <is>
+          <t>Task detail page at /tasks/[id]: Core (Task Number, Title, Client, Entity, Department, Service, Priority, Status, Source, Created) plus related data that already exists - the Engagement for this entity/service pairing (billing structure, engagement start, active/terminated), fetched separately from the task row to demonstrate real related-data loading, not just denormalized fields. Scoped to task:viewAll like the list (same known gap). PRD S18 describes a much larger screen (Client Instruction, AI Interpretation, Checklist, Attachments, Working Papers, Time, Comments, Client Communication, Review, Activity Timeline) - almost none of which exists yet (AI intake, attachments, time tracking, comments, review, and activity timeline are all separate later days/phases); this page adds each section as its own day builds it, rather than stubbing placeholders now. Also added GET /api/tasks/[id] (same route pattern as Client/Entity/Service) as the natural attachment point for status/assignment mutations once those days land. Unit/API + E2E tests cover the happy path, not-found, permission scoping, and auth.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="82.05" customHeight="1" s="9">
       <c r="A49" s="11" t="n">
@@ -8909,13 +8913,19 @@
       <c r="C33" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="D33" s="11" t="n"/>
+      <c r="D33" s="11" t="n">
+        <v>47</v>
+      </c>
       <c r="E33" s="11" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F33" s="11" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Task workspace with core fields and related Engagement data; grows section by section as later days (checklist, comments, attachments, etc.) land (see Daily Plan Day 47).</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="9">
       <c r="A34" s="11" t="inlineStr">

</xml_diff>